<commit_message>
Refactor digraph analysis & diagram FP
- Restructure digraph analysis and diagram generation APIs.
- cDigraphAnalysis was rewritten (new private data, SCC via dfSC, kernel construction, transitive-closure and getters) and now exposes organized Graph/Kernel tables, node/group getters and edge builders.
- cDiagramFP updated to use the new analysis API (GraphTable/KernelTable, getDigraph/getNodesTable, buildDigraph) and to return MATLAB digraph objects for visualization; node weight/topology handling adjusted.
- cDigraph now consumes info.getDigraph for building plot objects.
- ProductiveDiagram switched logger from cTaesLab to cMessageLogger and added an early return.
- Several legacy numeric helpers were removed (inverseMatrixOperator.m, npinv.m, nplu.m, sminv.m, topologicalOrder.m).
- Minor docs/comments updated.
</commit_message>
<xml_diff>
--- a/Examples/orcvcr/orcvcr_model.xlsx
+++ b/Examples/orcvcr/orcvcr_model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ctorr\Documents\Proyectos\TaesLab\Examples\orcvcr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1838FABF-A869-4526-924B-CDA499E9086F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4A5A24-B3F8-4D4C-8FAC-CC3D631BCBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="765" windowWidth="22965" windowHeight="14700" firstSheet="2" activeTab="4" xr2:uid="{E29BBF69-888A-4B0D-A36F-5F6BD99DC033}"/>
+    <workbookView xWindow="9255" yWindow="780" windowWidth="18630" windowHeight="14700" activeTab="3" xr2:uid="{E29BBF69-888A-4B0D-A36F-5F6BD99DC033}"/>
   </bookViews>
   <sheets>
     <sheet name="Physical Diagram" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,6 @@
     <sheet name="WasteAllocation" sheetId="8" r:id="rId8"/>
     <sheet name="ResourcesCost" sheetId="9" r:id="rId9"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId10"/>
-  </externalReferences>
   <definedNames>
     <definedName name="DATOS" localSheetId="4">Exergy!#REF!</definedName>
     <definedName name="tgas_fmt" localSheetId="5">Format!$A$1:$D$7</definedName>
@@ -66,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="89">
   <si>
     <t>Flows</t>
   </si>
@@ -327,6 +324,12 @@
   </si>
   <si>
     <t>WN0</t>
+  </si>
+  <si>
+    <t>TA30</t>
+  </si>
+  <si>
+    <t>TA30V</t>
   </si>
 </sst>
 </file>
@@ -405,23 +408,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>504826</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>219076</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>137195</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06948033-CC19-4A05-36F6-009C3DB8F861}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBE3C8C7-9245-6770-EE35-61B156C9397C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -444,8 +447,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1847850" y="180975"/>
-          <a:ext cx="5553075" cy="5048250"/>
+          <a:off x="1266826" y="247650"/>
+          <a:ext cx="8096250" cy="6176045"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -465,126 +468,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="REF"/>
-      <sheetName val="ETAT75"/>
-      <sheetName val="ETAC75"/>
-      <sheetName val="TCND35"/>
-      <sheetName val="TBLR85"/>
-      <sheetName val="WN200"/>
-      <sheetName val="Exergy"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="A1" t="str">
-            <v>key</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>B1</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>B2</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>B3</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>B4</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>B5</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>B6</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>B7</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>B8</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>WT</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>WC</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>WP</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>QBLR</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>QEVP</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>WN</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>QCND</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>QEXP</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5">
-        <row r="2">
-          <cell r="G2">
-            <v>1178</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="6"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1332,13 +1215,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C71C192-3DC3-406B-9DFF-73A67AE08F6E}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="str">
-        <f>[1]REF!A1</f>
-        <v>key</v>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>19</v>
       </c>
       <c r="B1" t="s">
         <v>78</v>
@@ -1361,11 +1243,16 @@
       <c r="H1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="str">
-        <f>[1]REF!A2</f>
-        <v>B1</v>
+      <c r="I1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>21</v>
       </c>
       <c r="B2">
         <v>684.6</v>
@@ -1388,11 +1275,16 @@
       <c r="H2">
         <v>1178</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="str">
-        <f>[1]REF!A3</f>
-        <v>B2</v>
+      <c r="I2">
+        <v>672</v>
+      </c>
+      <c r="J2">
+        <v>937.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
       </c>
       <c r="B3">
         <v>349.7</v>
@@ -1415,11 +1307,16 @@
       <c r="H3">
         <v>601.4</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="str">
-        <f>[1]REF!A4</f>
-        <v>B3</v>
+      <c r="I3">
+        <v>343.2</v>
+      </c>
+      <c r="J3">
+        <v>478.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
       </c>
       <c r="B4">
         <v>273.8</v>
@@ -1442,11 +1339,16 @@
       <c r="H4">
         <v>471</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="str">
-        <f>[1]REF!A5</f>
-        <v>B4</v>
+      <c r="I4">
+        <v>268.8</v>
+      </c>
+      <c r="J4">
+        <v>374.9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
       </c>
       <c r="B5">
         <v>287.89999999999998</v>
@@ -1469,11 +1371,16 @@
       <c r="H5">
         <v>495.1</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="str">
-        <f>[1]REF!A6</f>
-        <v>B5</v>
+      <c r="I5">
+        <v>282.60000000000002</v>
+      </c>
+      <c r="J5">
+        <v>394.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>25</v>
       </c>
       <c r="B6">
         <v>193.5</v>
@@ -1496,11 +1403,16 @@
       <c r="H6">
         <v>193.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="str">
-        <f>[1]REF!A7</f>
-        <v>B6</v>
+      <c r="I6">
+        <v>193.5</v>
+      </c>
+      <c r="J6">
+        <v>276.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
       </c>
       <c r="B7">
         <v>167.2</v>
@@ -1523,11 +1435,16 @@
       <c r="H7">
         <v>167.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="str">
-        <f>[1]REF!A8</f>
-        <v>B7</v>
+      <c r="I7">
+        <v>167.2</v>
+      </c>
+      <c r="J7">
+        <v>239.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
       </c>
       <c r="B8">
         <v>55.19</v>
@@ -1550,11 +1467,16 @@
       <c r="H8">
         <v>55.19</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="str">
-        <f>[1]REF!A9</f>
-        <v>B8</v>
+      <c r="I8">
+        <v>55.19</v>
+      </c>
+      <c r="J8">
+        <v>78.91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
       </c>
       <c r="B9">
         <v>240.8</v>
@@ -1577,11 +1499,16 @@
       <c r="H9">
         <v>240.8</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="str">
-        <f>[1]REF!A10</f>
-        <v>WT</v>
+      <c r="I9">
+        <v>240.8</v>
+      </c>
+      <c r="J9">
+        <v>344.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>29</v>
       </c>
       <c r="B10">
         <v>271.89999999999998</v>
@@ -1604,11 +1531,16 @@
       <c r="H10">
         <v>467.6</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="str">
-        <f>[1]REF!A11</f>
-        <v>WC</v>
+      <c r="I10">
+        <v>266.89999999999998</v>
+      </c>
+      <c r="J10">
+        <v>372.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>30</v>
       </c>
       <c r="B11">
         <v>230</v>
@@ -1631,11 +1563,16 @@
       <c r="H11">
         <v>230</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="str">
-        <f>[1]REF!A12</f>
-        <v>WP</v>
+      <c r="I11">
+        <v>230</v>
+      </c>
+      <c r="J11">
+        <v>328.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>31</v>
       </c>
       <c r="B12">
         <v>16.420000000000002</v>
@@ -1658,11 +1595,16 @@
       <c r="H12">
         <v>28.25</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="str">
-        <f>[1]REF!A13</f>
-        <v>QBLR</v>
+      <c r="I12">
+        <v>16.12</v>
+      </c>
+      <c r="J12">
+        <v>22.48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>53</v>
       </c>
       <c r="B13">
         <v>545.79999999999995</v>
@@ -1685,11 +1627,16 @@
       <c r="H13">
         <v>938.8</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="str">
-        <f>[1]REF!A14</f>
-        <v>QEVP</v>
+      <c r="I13">
+        <v>534.6</v>
+      </c>
+      <c r="J13">
+        <v>745.6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
       </c>
       <c r="B14">
         <v>42.96</v>
@@ -1712,11 +1659,16 @@
       <c r="H14">
         <v>42.96</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="str">
-        <f>[1]REF!A15</f>
-        <v>WN</v>
+      <c r="I14">
+        <v>35.090000000000003</v>
+      </c>
+      <c r="J14">
+        <v>50.17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>33</v>
       </c>
       <c r="B15">
         <v>20</v>
@@ -1739,11 +1691,16 @@
       <c r="H15">
         <v>200</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="str">
-        <f>[1]REF!A16</f>
-        <v>QCND</v>
+      <c r="I15">
+        <v>20</v>
+      </c>
+      <c r="J15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>54</v>
       </c>
       <c r="B16">
         <f>B3+B9-B4-B6</f>
@@ -1773,11 +1730,18 @@
         <f>H3+H9-H4-H6</f>
         <v>177.70000000000005</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="str">
-        <f>[1]REF!A17</f>
-        <v>QEXP</v>
+      <c r="I16">
+        <f>I3+I9-I4-I6</f>
+        <v>121.69999999999999</v>
+      </c>
+      <c r="J16">
+        <f>J3+J9-J4-J6</f>
+        <v>171.49999999999994</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>72</v>
       </c>
       <c r="B17">
         <f>B6-B7</f>
@@ -1806,6 +1770,14 @@
       <c r="H17">
         <f>H6-H7</f>
         <v>26.300000000000011</v>
+      </c>
+      <c r="I17">
+        <f>I6-I7</f>
+        <v>26.300000000000011</v>
+      </c>
+      <c r="J17">
+        <f>J6-J7</f>
+        <v>37.599999999999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>